<commit_message>
slight changes and new execution
</commit_message>
<xml_diff>
--- a/code/Created Files for Analysis/bip_levels_2006_2022.xlsx
+++ b/code/Created Files for Analysis/bip_levels_2006_2022.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2001"/>
+  <dimension ref="A1:D2018"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -34995,1458 +34995,1764 @@
     <row r="1921">
       <c r="A1921" t="inlineStr">
         <is>
-          <t>VNM</t>
+          <t>VEN</t>
         </is>
       </c>
       <c r="B1921" t="inlineStr">
         <is>
-          <t>Viet Nam</t>
+          <t>Venezuela, RB</t>
         </is>
       </c>
       <c r="C1921" t="n">
         <v>2006</v>
       </c>
       <c r="D1921" t="n">
-        <v>139658819217.11</v>
+        <v>114086845431.651</v>
       </c>
     </row>
     <row r="1922">
       <c r="A1922" t="inlineStr">
         <is>
-          <t>VNM</t>
+          <t>VEN</t>
         </is>
       </c>
       <c r="B1922" t="inlineStr">
         <is>
-          <t>Viet Nam</t>
+          <t>Venezuela, RB</t>
         </is>
       </c>
       <c r="C1922" t="n">
         <v>2007</v>
       </c>
       <c r="D1922" t="n">
-        <v>149615800998.3645</v>
+        <v>124133632211.346</v>
       </c>
     </row>
     <row r="1923">
       <c r="A1923" t="inlineStr">
         <is>
-          <t>VNM</t>
+          <t>VEN</t>
         </is>
       </c>
       <c r="B1923" t="inlineStr">
         <is>
-          <t>Viet Nam</t>
+          <t>Venezuela, RB</t>
         </is>
       </c>
       <c r="C1923" t="n">
         <v>2008</v>
       </c>
       <c r="D1923" t="n">
-        <v>158086705343.2754</v>
+        <v>130608228136.038</v>
       </c>
     </row>
     <row r="1924">
       <c r="A1924" t="inlineStr">
         <is>
-          <t>VNM</t>
+          <t>VEN</t>
         </is>
       </c>
       <c r="B1924" t="inlineStr">
         <is>
-          <t>Viet Nam</t>
+          <t>Venezuela, RB</t>
         </is>
       </c>
       <c r="C1924" t="n">
         <v>2009</v>
       </c>
       <c r="D1924" t="n">
-        <v>166620063722.2913</v>
+        <v>126589513424.16</v>
       </c>
     </row>
     <row r="1925">
       <c r="A1925" t="inlineStr">
         <is>
-          <t>VNM</t>
+          <t>VEN</t>
         </is>
       </c>
       <c r="B1925" t="inlineStr">
         <is>
-          <t>Viet Nam</t>
+          <t>Venezuela, RB</t>
         </is>
       </c>
       <c r="C1925" t="n">
         <v>2010</v>
       </c>
       <c r="D1925" t="n">
-        <v>177322478338.4043</v>
+        <v>124580156068.221</v>
       </c>
     </row>
     <row r="1926">
       <c r="A1926" t="inlineStr">
         <is>
-          <t>VNM</t>
+          <t>VEN</t>
         </is>
       </c>
       <c r="B1926" t="inlineStr">
         <is>
-          <t>Viet Nam</t>
+          <t>Venezuela, RB</t>
         </is>
       </c>
       <c r="C1926" t="n">
         <v>2011</v>
       </c>
       <c r="D1926" t="n">
-        <v>188694468366.2676</v>
+        <v>129715180422.288</v>
       </c>
     </row>
     <row r="1927">
       <c r="A1927" t="inlineStr">
         <is>
-          <t>VNM</t>
+          <t>VEN</t>
         </is>
       </c>
       <c r="B1927" t="inlineStr">
         <is>
-          <t>Viet Nam</t>
+          <t>Venezuela, RB</t>
         </is>
       </c>
       <c r="C1927" t="n">
         <v>2012</v>
       </c>
       <c r="D1927" t="n">
-        <v>199081239731.6883</v>
+        <v>137082824060.731</v>
       </c>
     </row>
     <row r="1928">
       <c r="A1928" t="inlineStr">
         <is>
-          <t>VNM</t>
+          <t>VEN</t>
         </is>
       </c>
       <c r="B1928" t="inlineStr">
         <is>
-          <t>Viet Nam</t>
+          <t>Venezuela, RB</t>
         </is>
       </c>
       <c r="C1928" t="n">
         <v>2013</v>
       </c>
       <c r="D1928" t="n">
-        <v>210137237901.3887</v>
+        <v>138868919488.232</v>
       </c>
     </row>
     <row r="1929">
       <c r="A1929" t="inlineStr">
         <is>
-          <t>VNM</t>
+          <t>VEN</t>
         </is>
       </c>
       <c r="B1929" t="inlineStr">
         <is>
-          <t>Viet Nam</t>
+          <t>Venezuela, RB</t>
         </is>
       </c>
       <c r="C1929" t="n">
         <v>2014</v>
       </c>
       <c r="D1929" t="n">
-        <v>223632762207.5602</v>
+        <v>133510633205.728</v>
       </c>
     </row>
     <row r="1930">
       <c r="A1930" t="inlineStr">
         <is>
-          <t>VNM</t>
+          <t>VEN</t>
         </is>
       </c>
       <c r="B1930" t="inlineStr">
         <is>
-          <t>Viet Nam</t>
+          <t>Venezuela, RB</t>
         </is>
       </c>
       <c r="C1930" t="n">
         <v>2015</v>
       </c>
       <c r="D1930" t="n">
-        <v>239258328381.7414</v>
+        <v>125249941853.534</v>
       </c>
     </row>
     <row r="1931">
       <c r="A1931" t="inlineStr">
         <is>
-          <t>VNM</t>
+          <t>VEN</t>
         </is>
       </c>
       <c r="B1931" t="inlineStr">
         <is>
-          <t>Viet Nam</t>
+          <t>Venezuela, RB</t>
         </is>
       </c>
       <c r="C1931" t="n">
         <v>2016</v>
       </c>
       <c r="D1931" t="n">
-        <v>255264731908.124</v>
+        <v>103816796723.518</v>
       </c>
     </row>
     <row r="1932">
       <c r="A1932" t="inlineStr">
         <is>
-          <t>VNM</t>
+          <t>VEN</t>
         </is>
       </c>
       <c r="B1932" t="inlineStr">
         <is>
-          <t>Viet Nam</t>
+          <t>Venezuela, RB</t>
         </is>
       </c>
       <c r="C1932" t="n">
         <v>2017</v>
       </c>
       <c r="D1932" t="n">
-        <v>272980590259.1872</v>
+        <v>87518675947.5676</v>
       </c>
     </row>
     <row r="1933">
       <c r="A1933" t="inlineStr">
         <is>
-          <t>VNM</t>
+          <t>VEN</t>
         </is>
       </c>
       <c r="B1933" t="inlineStr">
         <is>
-          <t>Viet Nam</t>
+          <t>Venezuela, RB</t>
         </is>
       </c>
       <c r="C1933" t="n">
         <v>2018</v>
       </c>
       <c r="D1933" t="n">
-        <v>293358610036.8409</v>
+        <v>70327507457.86681</v>
       </c>
     </row>
     <row r="1934">
       <c r="A1934" t="inlineStr">
         <is>
-          <t>VNM</t>
+          <t>VEN</t>
         </is>
       </c>
       <c r="B1934" t="inlineStr">
         <is>
-          <t>Viet Nam</t>
+          <t>Venezuela, RB</t>
         </is>
       </c>
       <c r="C1934" t="n">
         <v>2019</v>
       </c>
       <c r="D1934" t="n">
-        <v>314947640805.6011</v>
+        <v>50903719683.7893</v>
       </c>
     </row>
     <row r="1935">
       <c r="A1935" t="inlineStr">
         <is>
-          <t>VNM</t>
+          <t>VEN</t>
         </is>
       </c>
       <c r="B1935" t="inlineStr">
         <is>
-          <t>Viet Nam</t>
+          <t>Venezuela, RB</t>
         </is>
       </c>
       <c r="C1935" t="n">
         <v>2020</v>
       </c>
       <c r="D1935" t="n">
-        <v>323972192107.0652</v>
+        <v>35721908550.0276</v>
       </c>
     </row>
     <row r="1936">
       <c r="A1936" t="inlineStr">
         <is>
-          <t>VNM</t>
+          <t>VEN</t>
         </is>
       </c>
       <c r="B1936" t="inlineStr">
         <is>
-          <t>Viet Nam</t>
+          <t>Venezuela, RB</t>
         </is>
       </c>
       <c r="C1936" t="n">
         <v>2021</v>
       </c>
       <c r="D1936" t="n">
-        <v>332270947495.8008</v>
+        <v>35945170478.4652</v>
       </c>
     </row>
     <row r="1937">
       <c r="A1937" t="inlineStr">
         <is>
-          <t>VNM</t>
+          <t>VEN</t>
         </is>
       </c>
       <c r="B1937" t="inlineStr">
         <is>
-          <t>Viet Nam</t>
+          <t>Venezuela, RB</t>
         </is>
       </c>
       <c r="C1937" t="n">
         <v>2022</v>
       </c>
       <c r="D1937" t="n">
-        <v>358918387605.51</v>
+        <v>38847575548.155</v>
       </c>
     </row>
     <row r="1938">
       <c r="A1938" t="inlineStr">
         <is>
-          <t>YEM</t>
+          <t>VNM</t>
         </is>
       </c>
       <c r="B1938" t="inlineStr">
         <is>
-          <t>Yemen, Rep.</t>
+          <t>Viet Nam</t>
         </is>
       </c>
       <c r="C1938" t="n">
         <v>2006</v>
       </c>
       <c r="D1938" t="n">
-        <v>52612232709.0259</v>
+        <v>139658819217.11</v>
       </c>
     </row>
     <row r="1939">
       <c r="A1939" t="inlineStr">
         <is>
-          <t>YEM</t>
+          <t>VNM</t>
         </is>
       </c>
       <c r="B1939" t="inlineStr">
         <is>
-          <t>Yemen, Rep.</t>
+          <t>Viet Nam</t>
         </is>
       </c>
       <c r="C1939" t="n">
         <v>2007</v>
       </c>
       <c r="D1939" t="n">
-        <v>54368654194.08662</v>
+        <v>149615800998.3645</v>
       </c>
     </row>
     <row r="1940">
       <c r="A1940" t="inlineStr">
         <is>
-          <t>YEM</t>
+          <t>VNM</t>
         </is>
       </c>
       <c r="B1940" t="inlineStr">
         <is>
-          <t>Yemen, Rep.</t>
+          <t>Viet Nam</t>
         </is>
       </c>
       <c r="C1940" t="n">
         <v>2008</v>
       </c>
       <c r="D1940" t="n">
-        <v>56351788625.78867</v>
+        <v>158086705343.2754</v>
       </c>
     </row>
     <row r="1941">
       <c r="A1941" t="inlineStr">
         <is>
-          <t>YEM</t>
+          <t>VNM</t>
         </is>
       </c>
       <c r="B1941" t="inlineStr">
         <is>
-          <t>Yemen, Rep.</t>
+          <t>Viet Nam</t>
         </is>
       </c>
       <c r="C1941" t="n">
         <v>2009</v>
       </c>
       <c r="D1941" t="n">
-        <v>58530478110.36378</v>
+        <v>166620063722.2913</v>
       </c>
     </row>
     <row r="1942">
       <c r="A1942" t="inlineStr">
         <is>
-          <t>YEM</t>
+          <t>VNM</t>
         </is>
       </c>
       <c r="B1942" t="inlineStr">
         <is>
-          <t>Yemen, Rep.</t>
+          <t>Viet Nam</t>
         </is>
       </c>
       <c r="C1942" t="n">
         <v>2010</v>
       </c>
       <c r="D1942" t="n">
-        <v>63038675246.18078</v>
+        <v>177322478338.4043</v>
       </c>
     </row>
     <row r="1943">
       <c r="A1943" t="inlineStr">
         <is>
-          <t>YEM</t>
+          <t>VNM</t>
         </is>
       </c>
       <c r="B1943" t="inlineStr">
         <is>
-          <t>Yemen, Rep.</t>
+          <t>Viet Nam</t>
         </is>
       </c>
       <c r="C1943" t="n">
         <v>2011</v>
       </c>
       <c r="D1943" t="n">
-        <v>55023372684.39548</v>
+        <v>188694468366.2676</v>
       </c>
     </row>
     <row r="1944">
       <c r="A1944" t="inlineStr">
         <is>
-          <t>YEM</t>
+          <t>VNM</t>
         </is>
       </c>
       <c r="B1944" t="inlineStr">
         <is>
-          <t>Yemen, Rep.</t>
+          <t>Viet Nam</t>
         </is>
       </c>
       <c r="C1944" t="n">
         <v>2012</v>
       </c>
       <c r="D1944" t="n">
-        <v>56340076605.58898</v>
+        <v>199081239731.6883</v>
       </c>
     </row>
     <row r="1945">
       <c r="A1945" t="inlineStr">
         <is>
-          <t>YEM</t>
+          <t>VNM</t>
         </is>
       </c>
       <c r="B1945" t="inlineStr">
         <is>
-          <t>Yemen, Rep.</t>
+          <t>Viet Nam</t>
         </is>
       </c>
       <c r="C1945" t="n">
         <v>2013</v>
       </c>
       <c r="D1945" t="n">
-        <v>59057650942.74328</v>
+        <v>210137237901.3887</v>
       </c>
     </row>
     <row r="1946">
       <c r="A1946" t="inlineStr">
         <is>
-          <t>YEM</t>
+          <t>VNM</t>
         </is>
       </c>
       <c r="B1946" t="inlineStr">
         <is>
-          <t>Yemen, Rep.</t>
+          <t>Viet Nam</t>
         </is>
       </c>
       <c r="C1946" t="n">
         <v>2014</v>
       </c>
       <c r="D1946" t="n">
-        <v>58946214923.89937</v>
+        <v>223632762207.5602</v>
       </c>
     </row>
     <row r="1947">
       <c r="A1947" t="inlineStr">
         <is>
-          <t>YEM</t>
+          <t>VNM</t>
         </is>
       </c>
       <c r="B1947" t="inlineStr">
         <is>
-          <t>Yemen, Rep.</t>
+          <t>Viet Nam</t>
         </is>
       </c>
       <c r="C1947" t="n">
         <v>2015</v>
       </c>
       <c r="D1947" t="n">
-        <v>42444489522.23031</v>
+        <v>239258328381.7414</v>
       </c>
     </row>
     <row r="1948">
       <c r="A1948" t="inlineStr">
         <is>
-          <t>YEM</t>
+          <t>VNM</t>
         </is>
       </c>
       <c r="B1948" t="inlineStr">
         <is>
-          <t>Yemen, Rep.</t>
+          <t>Viet Nam</t>
         </is>
       </c>
       <c r="C1948" t="n">
         <v>2016</v>
       </c>
       <c r="D1948" t="n">
-        <v>38465266075.76577</v>
+        <v>255264731908.124</v>
       </c>
     </row>
     <row r="1949">
       <c r="A1949" t="inlineStr">
         <is>
-          <t>YEM</t>
+          <t>VNM</t>
         </is>
       </c>
       <c r="B1949" t="inlineStr">
         <is>
-          <t>Yemen, Rep.</t>
+          <t>Viet Nam</t>
         </is>
       </c>
       <c r="C1949" t="n">
         <v>2017</v>
       </c>
       <c r="D1949" t="n">
-        <v>36514386388.46739</v>
+        <v>272980590259.1872</v>
       </c>
     </row>
     <row r="1950">
       <c r="A1950" t="inlineStr">
         <is>
-          <t>YEM</t>
+          <t>VNM</t>
         </is>
       </c>
       <c r="B1950" t="inlineStr">
         <is>
-          <t>Yemen, Rep.</t>
+          <t>Viet Nam</t>
         </is>
       </c>
       <c r="C1950" t="n">
         <v>2018</v>
       </c>
       <c r="D1950" t="n">
-        <v>36789138007.96674</v>
+        <v>293358610036.8409</v>
       </c>
     </row>
     <row r="1951">
       <c r="A1951" t="inlineStr">
         <is>
-          <t>ZAF</t>
+          <t>VNM</t>
         </is>
       </c>
       <c r="B1951" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Viet Nam</t>
         </is>
       </c>
       <c r="C1951" t="n">
-        <v>2006</v>
+        <v>2019</v>
       </c>
       <c r="D1951" t="n">
-        <v>282539679229.8738</v>
+        <v>314947640805.6011</v>
       </c>
     </row>
     <row r="1952">
       <c r="A1952" t="inlineStr">
         <is>
-          <t>ZAF</t>
+          <t>VNM</t>
         </is>
       </c>
       <c r="B1952" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Viet Nam</t>
         </is>
       </c>
       <c r="C1952" t="n">
-        <v>2007</v>
+        <v>2020</v>
       </c>
       <c r="D1952" t="n">
-        <v>297685145427.0811</v>
+        <v>323972192107.0652</v>
       </c>
     </row>
     <row r="1953">
       <c r="A1953" t="inlineStr">
         <is>
-          <t>ZAF</t>
+          <t>VNM</t>
         </is>
       </c>
       <c r="B1953" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Viet Nam</t>
         </is>
       </c>
       <c r="C1953" t="n">
-        <v>2008</v>
+        <v>2021</v>
       </c>
       <c r="D1953" t="n">
-        <v>307184409060.7409</v>
+        <v>332270947495.8008</v>
       </c>
     </row>
     <row r="1954">
       <c r="A1954" t="inlineStr">
         <is>
-          <t>ZAF</t>
+          <t>VNM</t>
         </is>
       </c>
       <c r="B1954" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Viet Nam</t>
         </is>
       </c>
       <c r="C1954" t="n">
-        <v>2009</v>
+        <v>2022</v>
       </c>
       <c r="D1954" t="n">
-        <v>302459639039.7778</v>
+        <v>358918387605.51</v>
       </c>
     </row>
     <row r="1955">
       <c r="A1955" t="inlineStr">
         <is>
-          <t>ZAF</t>
+          <t>YEM</t>
         </is>
       </c>
       <c r="B1955" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Yemen, Rep.</t>
         </is>
       </c>
       <c r="C1955" t="n">
-        <v>2010</v>
+        <v>2006</v>
       </c>
       <c r="D1955" t="n">
-        <v>311653604140.2694</v>
+        <v>52612232709.0259</v>
       </c>
     </row>
     <row r="1956">
       <c r="A1956" t="inlineStr">
         <is>
-          <t>ZAF</t>
+          <t>YEM</t>
         </is>
       </c>
       <c r="B1956" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Yemen, Rep.</t>
         </is>
       </c>
       <c r="C1956" t="n">
-        <v>2011</v>
+        <v>2007</v>
       </c>
       <c r="D1956" t="n">
-        <v>321528523981.7023</v>
+        <v>54368654194.08662</v>
       </c>
     </row>
     <row r="1957">
       <c r="A1957" t="inlineStr">
         <is>
-          <t>ZAF</t>
+          <t>YEM</t>
         </is>
       </c>
       <c r="B1957" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Yemen, Rep.</t>
         </is>
       </c>
       <c r="C1957" t="n">
-        <v>2012</v>
+        <v>2008</v>
       </c>
       <c r="D1957" t="n">
-        <v>329233094599.2629</v>
+        <v>56351788625.78867</v>
       </c>
     </row>
     <row r="1958">
       <c r="A1958" t="inlineStr">
         <is>
-          <t>ZAF</t>
+          <t>YEM</t>
         </is>
       </c>
       <c r="B1958" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Yemen, Rep.</t>
         </is>
       </c>
       <c r="C1958" t="n">
-        <v>2013</v>
+        <v>2009</v>
       </c>
       <c r="D1958" t="n">
-        <v>337416077838.1514</v>
+        <v>58530478110.36378</v>
       </c>
     </row>
     <row r="1959">
       <c r="A1959" t="inlineStr">
         <is>
-          <t>ZAF</t>
+          <t>YEM</t>
         </is>
       </c>
       <c r="B1959" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Yemen, Rep.</t>
         </is>
       </c>
       <c r="C1959" t="n">
-        <v>2014</v>
+        <v>2010</v>
       </c>
       <c r="D1959" t="n">
-        <v>342186555600.7309</v>
+        <v>63038675246.18078</v>
       </c>
     </row>
     <row r="1960">
       <c r="A1960" t="inlineStr">
         <is>
-          <t>ZAF</t>
+          <t>YEM</t>
         </is>
       </c>
       <c r="B1960" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Yemen, Rep.</t>
         </is>
       </c>
       <c r="C1960" t="n">
-        <v>2015</v>
+        <v>2011</v>
       </c>
       <c r="D1960" t="n">
-        <v>346709790458.563</v>
+        <v>55023372684.39548</v>
       </c>
     </row>
     <row r="1961">
       <c r="A1961" t="inlineStr">
         <is>
-          <t>ZAF</t>
+          <t>YEM</t>
         </is>
       </c>
       <c r="B1961" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Yemen, Rep.</t>
         </is>
       </c>
       <c r="C1961" t="n">
-        <v>2016</v>
+        <v>2012</v>
       </c>
       <c r="D1961" t="n">
-        <v>349013858372.6254</v>
+        <v>56340076605.58898</v>
       </c>
     </row>
     <row r="1962">
       <c r="A1962" t="inlineStr">
         <is>
-          <t>ZAF</t>
+          <t>YEM</t>
         </is>
       </c>
       <c r="B1962" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Yemen, Rep.</t>
         </is>
       </c>
       <c r="C1962" t="n">
-        <v>2017</v>
+        <v>2013</v>
       </c>
       <c r="D1962" t="n">
-        <v>353055253705.8817</v>
+        <v>59057650942.74328</v>
       </c>
     </row>
     <row r="1963">
       <c r="A1963" t="inlineStr">
         <is>
-          <t>ZAF</t>
+          <t>YEM</t>
         </is>
       </c>
       <c r="B1963" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Yemen, Rep.</t>
         </is>
       </c>
       <c r="C1963" t="n">
-        <v>2018</v>
+        <v>2014</v>
       </c>
       <c r="D1963" t="n">
-        <v>358551560864.8784</v>
+        <v>58946214923.89937</v>
       </c>
     </row>
     <row r="1964">
       <c r="A1964" t="inlineStr">
         <is>
-          <t>ZAF</t>
+          <t>YEM</t>
         </is>
       </c>
       <c r="B1964" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Yemen, Rep.</t>
         </is>
       </c>
       <c r="C1964" t="n">
-        <v>2019</v>
+        <v>2015</v>
       </c>
       <c r="D1964" t="n">
-        <v>359483563933.709</v>
+        <v>42444489522.23031</v>
       </c>
     </row>
     <row r="1965">
       <c r="A1965" t="inlineStr">
         <is>
-          <t>ZAF</t>
+          <t>YEM</t>
         </is>
       </c>
       <c r="B1965" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Yemen, Rep.</t>
         </is>
       </c>
       <c r="C1965" t="n">
-        <v>2020</v>
+        <v>2016</v>
       </c>
       <c r="D1965" t="n">
-        <v>338046271407.9034</v>
+        <v>38465266075.76577</v>
       </c>
     </row>
     <row r="1966">
       <c r="A1966" t="inlineStr">
         <is>
-          <t>ZAF</t>
+          <t>YEM</t>
         </is>
       </c>
       <c r="B1966" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Yemen, Rep.</t>
         </is>
       </c>
       <c r="C1966" t="n">
-        <v>2021</v>
+        <v>2017</v>
       </c>
       <c r="D1966" t="n">
-        <v>353944797356.9</v>
+        <v>36514386388.46739</v>
       </c>
     </row>
     <row r="1967">
       <c r="A1967" t="inlineStr">
         <is>
-          <t>ZAF</t>
+          <t>YEM</t>
         </is>
       </c>
       <c r="B1967" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Yemen, Rep.</t>
         </is>
       </c>
       <c r="C1967" t="n">
-        <v>2022</v>
+        <v>2018</v>
       </c>
       <c r="D1967" t="n">
-        <v>360706580601.809</v>
+        <v>36789138007.96674</v>
       </c>
     </row>
     <row r="1968">
       <c r="A1968" t="inlineStr">
         <is>
-          <t>ZMB</t>
+          <t>ZAF</t>
         </is>
       </c>
       <c r="B1968" t="inlineStr">
         <is>
-          <t>Zambia</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C1968" t="n">
         <v>2006</v>
       </c>
       <c r="D1968" t="n">
-        <v>11748243095.77287</v>
+        <v>282539679229.8738</v>
       </c>
     </row>
     <row r="1969">
       <c r="A1969" t="inlineStr">
         <is>
-          <t>ZMB</t>
+          <t>ZAF</t>
         </is>
       </c>
       <c r="B1969" t="inlineStr">
         <is>
-          <t>Zambia</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C1969" t="n">
         <v>2007</v>
       </c>
       <c r="D1969" t="n">
-        <v>12729507610.19313</v>
+        <v>297685145427.0811</v>
       </c>
     </row>
     <row r="1970">
       <c r="A1970" t="inlineStr">
         <is>
-          <t>ZMB</t>
+          <t>ZAF</t>
         </is>
       </c>
       <c r="B1970" t="inlineStr">
         <is>
-          <t>Zambia</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C1970" t="n">
         <v>2008</v>
       </c>
       <c r="D1970" t="n">
-        <v>13719086269.62596</v>
+        <v>307184409060.7409</v>
       </c>
     </row>
     <row r="1971">
       <c r="A1971" t="inlineStr">
         <is>
-          <t>ZMB</t>
+          <t>ZAF</t>
         </is>
       </c>
       <c r="B1971" t="inlineStr">
         <is>
-          <t>Zambia</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C1971" t="n">
         <v>2009</v>
       </c>
       <c r="D1971" t="n">
-        <v>14984033821.78684</v>
+        <v>302459639039.7778</v>
       </c>
     </row>
     <row r="1972">
       <c r="A1972" t="inlineStr">
         <is>
-          <t>ZMB</t>
+          <t>ZAF</t>
         </is>
       </c>
       <c r="B1972" t="inlineStr">
         <is>
-          <t>Zambia</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C1972" t="n">
         <v>2010</v>
       </c>
       <c r="D1972" t="n">
-        <v>16527123087.71631</v>
+        <v>311653604140.2694</v>
       </c>
     </row>
     <row r="1973">
       <c r="A1973" t="inlineStr">
         <is>
-          <t>ZMB</t>
+          <t>ZAF</t>
         </is>
       </c>
       <c r="B1973" t="inlineStr">
         <is>
-          <t>Zambia</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C1973" t="n">
         <v>2011</v>
       </c>
       <c r="D1973" t="n">
-        <v>17446791765.2459</v>
+        <v>321528523981.7023</v>
       </c>
     </row>
     <row r="1974">
       <c r="A1974" t="inlineStr">
         <is>
-          <t>ZMB</t>
+          <t>ZAF</t>
         </is>
       </c>
       <c r="B1974" t="inlineStr">
         <is>
-          <t>Zambia</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C1974" t="n">
         <v>2012</v>
       </c>
       <c r="D1974" t="n">
-        <v>18772328031.85786</v>
+        <v>329233094599.2629</v>
       </c>
     </row>
     <row r="1975">
       <c r="A1975" t="inlineStr">
         <is>
-          <t>ZMB</t>
+          <t>ZAF</t>
         </is>
       </c>
       <c r="B1975" t="inlineStr">
         <is>
-          <t>Zambia</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C1975" t="n">
         <v>2013</v>
       </c>
       <c r="D1975" t="n">
-        <v>19721688163.38386</v>
+        <v>337416077838.1514</v>
       </c>
     </row>
     <row r="1976">
       <c r="A1976" t="inlineStr">
         <is>
-          <t>ZMB</t>
+          <t>ZAF</t>
         </is>
       </c>
       <c r="B1976" t="inlineStr">
         <is>
-          <t>Zambia</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C1976" t="n">
         <v>2014</v>
       </c>
       <c r="D1976" t="n">
-        <v>20648211567.06158</v>
+        <v>342186555600.7309</v>
       </c>
     </row>
     <row r="1977">
       <c r="A1977" t="inlineStr">
         <is>
-          <t>ZMB</t>
+          <t>ZAF</t>
         </is>
       </c>
       <c r="B1977" t="inlineStr">
         <is>
-          <t>Zambia</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C1977" t="n">
         <v>2015</v>
       </c>
       <c r="D1977" t="n">
-        <v>21251216798.77625</v>
+        <v>346709790458.563</v>
       </c>
     </row>
     <row r="1978">
       <c r="A1978" t="inlineStr">
         <is>
-          <t>ZMB</t>
+          <t>ZAF</t>
         </is>
       </c>
       <c r="B1978" t="inlineStr">
         <is>
-          <t>Zambia</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C1978" t="n">
         <v>2016</v>
       </c>
       <c r="D1978" t="n">
-        <v>22053807071.94368</v>
+        <v>349013858372.6254</v>
       </c>
     </row>
     <row r="1979">
       <c r="A1979" t="inlineStr">
         <is>
-          <t>ZMB</t>
+          <t>ZAF</t>
         </is>
       </c>
       <c r="B1979" t="inlineStr">
         <is>
-          <t>Zambia</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C1979" t="n">
         <v>2017</v>
       </c>
       <c r="D1979" t="n">
-        <v>22826646593.61689</v>
+        <v>353055253705.8817</v>
       </c>
     </row>
     <row r="1980">
       <c r="A1980" t="inlineStr">
         <is>
-          <t>ZMB</t>
+          <t>ZAF</t>
         </is>
       </c>
       <c r="B1980" t="inlineStr">
         <is>
-          <t>Zambia</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C1980" t="n">
         <v>2018</v>
       </c>
       <c r="D1980" t="n">
-        <v>23747586257.25117</v>
+        <v>358551560864.8784</v>
       </c>
     </row>
     <row r="1981">
       <c r="A1981" t="inlineStr">
         <is>
-          <t>ZMB</t>
+          <t>ZAF</t>
         </is>
       </c>
       <c r="B1981" t="inlineStr">
         <is>
-          <t>Zambia</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C1981" t="n">
         <v>2019</v>
       </c>
       <c r="D1981" t="n">
-        <v>24089861649.01546</v>
+        <v>359483563933.709</v>
       </c>
     </row>
     <row r="1982">
       <c r="A1982" t="inlineStr">
         <is>
-          <t>ZMB</t>
+          <t>ZAF</t>
         </is>
       </c>
       <c r="B1982" t="inlineStr">
         <is>
-          <t>Zambia</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C1982" t="n">
         <v>2020</v>
       </c>
       <c r="D1982" t="n">
-        <v>23418945736.89926</v>
+        <v>338046271407.9034</v>
       </c>
     </row>
     <row r="1983">
       <c r="A1983" t="inlineStr">
         <is>
-          <t>ZMB</t>
+          <t>ZAF</t>
         </is>
       </c>
       <c r="B1983" t="inlineStr">
         <is>
-          <t>Zambia</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C1983" t="n">
         <v>2021</v>
       </c>
       <c r="D1983" t="n">
-        <v>24879098746.62993</v>
+        <v>353944797356.9</v>
       </c>
     </row>
     <row r="1984">
       <c r="A1984" t="inlineStr">
         <is>
-          <t>ZMB</t>
+          <t>ZAF</t>
         </is>
       </c>
       <c r="B1984" t="inlineStr">
         <is>
-          <t>Zambia</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C1984" t="n">
         <v>2022</v>
       </c>
       <c r="D1984" t="n">
-        <v>26185157462.01585</v>
+        <v>360706580601.809</v>
       </c>
     </row>
     <row r="1985">
       <c r="A1985" t="inlineStr">
         <is>
-          <t>ZWE</t>
+          <t>ZMB</t>
         </is>
       </c>
       <c r="B1985" t="inlineStr">
         <is>
-          <t>Zimbabwe</t>
+          <t>Zambia</t>
         </is>
       </c>
       <c r="C1985" t="n">
         <v>2006</v>
       </c>
       <c r="D1985" t="n">
-        <v>13049672720.22442</v>
+        <v>11748243095.77287</v>
       </c>
     </row>
     <row r="1986">
       <c r="A1986" t="inlineStr">
         <is>
-          <t>ZWE</t>
+          <t>ZMB</t>
         </is>
       </c>
       <c r="B1986" t="inlineStr">
         <is>
-          <t>Zimbabwe</t>
+          <t>Zambia</t>
         </is>
       </c>
       <c r="C1986" t="n">
         <v>2007</v>
       </c>
       <c r="D1986" t="n">
-        <v>12572925524.81045</v>
+        <v>12729507610.19313</v>
       </c>
     </row>
     <row r="1987">
       <c r="A1987" t="inlineStr">
         <is>
-          <t>ZWE</t>
+          <t>ZMB</t>
         </is>
       </c>
       <c r="B1987" t="inlineStr">
         <is>
-          <t>Zimbabwe</t>
+          <t>Zambia</t>
         </is>
       </c>
       <c r="C1987" t="n">
         <v>2008</v>
       </c>
       <c r="D1987" t="n">
-        <v>10351422061.70757</v>
+        <v>13719086269.62596</v>
       </c>
     </row>
     <row r="1988">
       <c r="A1988" t="inlineStr">
         <is>
-          <t>ZWE</t>
+          <t>ZMB</t>
         </is>
       </c>
       <c r="B1988" t="inlineStr">
         <is>
-          <t>Zimbabwe</t>
+          <t>Zambia</t>
         </is>
       </c>
       <c r="C1988" t="n">
         <v>2009</v>
       </c>
       <c r="D1988" t="n">
-        <v>11595617444.66356</v>
+        <v>14984033821.78684</v>
       </c>
     </row>
     <row r="1989">
       <c r="A1989" t="inlineStr">
         <is>
-          <t>ZWE</t>
+          <t>ZMB</t>
         </is>
       </c>
       <c r="B1989" t="inlineStr">
         <is>
-          <t>Zimbabwe</t>
+          <t>Zambia</t>
         </is>
       </c>
       <c r="C1989" t="n">
         <v>2010</v>
       </c>
       <c r="D1989" t="n">
-        <v>14083116362.76866</v>
+        <v>16527123087.71631</v>
       </c>
     </row>
     <row r="1990">
       <c r="A1990" t="inlineStr">
         <is>
-          <t>ZWE</t>
+          <t>ZMB</t>
         </is>
       </c>
       <c r="B1990" t="inlineStr">
         <is>
-          <t>Zimbabwe</t>
+          <t>Zambia</t>
         </is>
       </c>
       <c r="C1990" t="n">
         <v>2011</v>
       </c>
       <c r="D1990" t="n">
-        <v>16142097162.99623</v>
+        <v>17446791765.2459</v>
       </c>
     </row>
     <row r="1991">
       <c r="A1991" t="inlineStr">
         <is>
-          <t>ZWE</t>
+          <t>ZMB</t>
         </is>
       </c>
       <c r="B1991" t="inlineStr">
         <is>
-          <t>Zimbabwe</t>
+          <t>Zambia</t>
         </is>
       </c>
       <c r="C1991" t="n">
         <v>2012</v>
       </c>
       <c r="D1991" t="n">
-        <v>18683650519.49866</v>
+        <v>18772328031.85786</v>
       </c>
     </row>
     <row r="1992">
       <c r="A1992" t="inlineStr">
         <is>
-          <t>ZWE</t>
+          <t>ZMB</t>
         </is>
       </c>
       <c r="B1992" t="inlineStr">
         <is>
-          <t>Zimbabwe</t>
+          <t>Zambia</t>
         </is>
       </c>
       <c r="C1992" t="n">
         <v>2013</v>
       </c>
       <c r="D1992" t="n">
-        <v>19280916546.44884</v>
+        <v>19721688163.38386</v>
       </c>
     </row>
     <row r="1993">
       <c r="A1993" t="inlineStr">
         <is>
-          <t>ZWE</t>
+          <t>ZMB</t>
         </is>
       </c>
       <c r="B1993" t="inlineStr">
         <is>
-          <t>Zimbabwe</t>
+          <t>Zambia</t>
         </is>
       </c>
       <c r="C1993" t="n">
         <v>2014</v>
       </c>
       <c r="D1993" t="n">
-        <v>19567149970.42023</v>
+        <v>20648211567.06158</v>
       </c>
     </row>
     <row r="1994">
       <c r="A1994" t="inlineStr">
         <is>
-          <t>ZWE</t>
+          <t>ZMB</t>
         </is>
       </c>
       <c r="B1994" t="inlineStr">
         <is>
-          <t>Zimbabwe</t>
+          <t>Zambia</t>
         </is>
       </c>
       <c r="C1994" t="n">
         <v>2015</v>
       </c>
       <c r="D1994" t="n">
-        <v>19963120600</v>
+        <v>21251216798.77625</v>
       </c>
     </row>
     <row r="1995">
       <c r="A1995" t="inlineStr">
         <is>
-          <t>ZWE</t>
+          <t>ZMB</t>
         </is>
       </c>
       <c r="B1995" t="inlineStr">
         <is>
-          <t>Zimbabwe</t>
+          <t>Zambia</t>
         </is>
       </c>
       <c r="C1995" t="n">
         <v>2016</v>
       </c>
       <c r="D1995" t="n">
-        <v>20142979412.31727</v>
+        <v>22053807071.94368</v>
       </c>
     </row>
     <row r="1996">
       <c r="A1996" t="inlineStr">
         <is>
-          <t>ZWE</t>
+          <t>ZMB</t>
         </is>
       </c>
       <c r="B1996" t="inlineStr">
         <is>
-          <t>Zimbabwe</t>
+          <t>Zambia</t>
         </is>
       </c>
       <c r="C1996" t="n">
         <v>2017</v>
       </c>
       <c r="D1996" t="n">
-        <v>20964866130.33335</v>
+        <v>22826646593.61689</v>
       </c>
     </row>
     <row r="1997">
       <c r="A1997" t="inlineStr">
         <is>
-          <t>ZWE</t>
+          <t>ZMB</t>
         </is>
       </c>
       <c r="B1997" t="inlineStr">
         <is>
-          <t>Zimbabwe</t>
+          <t>Zambia</t>
         </is>
       </c>
       <c r="C1997" t="n">
         <v>2018</v>
       </c>
       <c r="D1997" t="n">
-        <v>22015177994.7607</v>
+        <v>23747586257.25117</v>
       </c>
     </row>
     <row r="1998">
       <c r="A1998" t="inlineStr">
         <is>
-          <t>ZWE</t>
+          <t>ZMB</t>
         </is>
       </c>
       <c r="B1998" t="inlineStr">
         <is>
-          <t>Zimbabwe</t>
+          <t>Zambia</t>
         </is>
       </c>
       <c r="C1998" t="n">
         <v>2019</v>
       </c>
       <c r="D1998" t="n">
-        <v>20621078642.74352</v>
+        <v>24089861649.01546</v>
       </c>
     </row>
     <row r="1999">
       <c r="A1999" t="inlineStr">
         <is>
-          <t>ZWE</t>
+          <t>ZMB</t>
         </is>
       </c>
       <c r="B1999" t="inlineStr">
         <is>
-          <t>Zimbabwe</t>
+          <t>Zambia</t>
         </is>
       </c>
       <c r="C1999" t="n">
         <v>2020</v>
       </c>
       <c r="D1999" t="n">
-        <v>19009139108.24475</v>
+        <v>23418945736.89926</v>
       </c>
     </row>
     <row r="2000">
       <c r="A2000" t="inlineStr">
         <is>
-          <t>ZWE</t>
+          <t>ZMB</t>
         </is>
       </c>
       <c r="B2000" t="inlineStr">
         <is>
-          <t>Zimbabwe</t>
+          <t>Zambia</t>
         </is>
       </c>
       <c r="C2000" t="n">
         <v>2021</v>
       </c>
       <c r="D2000" t="n">
-        <v>20618836222.17532</v>
+        <v>24879098746.62993</v>
       </c>
     </row>
     <row r="2001">
       <c r="A2001" t="inlineStr">
         <is>
-          <t>ZWE</t>
+          <t>ZMB</t>
         </is>
       </c>
       <c r="B2001" t="inlineStr">
         <is>
-          <t>Zimbabwe</t>
+          <t>Zambia</t>
         </is>
       </c>
       <c r="C2001" t="n">
         <v>2022</v>
       </c>
       <c r="D2001" t="n">
+        <v>26185157462.01585</v>
+      </c>
+    </row>
+    <row r="2002">
+      <c r="A2002" t="inlineStr">
+        <is>
+          <t>ZWE</t>
+        </is>
+      </c>
+      <c r="B2002" t="inlineStr">
+        <is>
+          <t>Zimbabwe</t>
+        </is>
+      </c>
+      <c r="C2002" t="n">
+        <v>2006</v>
+      </c>
+      <c r="D2002" t="n">
+        <v>13049672720.22442</v>
+      </c>
+    </row>
+    <row r="2003">
+      <c r="A2003" t="inlineStr">
+        <is>
+          <t>ZWE</t>
+        </is>
+      </c>
+      <c r="B2003" t="inlineStr">
+        <is>
+          <t>Zimbabwe</t>
+        </is>
+      </c>
+      <c r="C2003" t="n">
+        <v>2007</v>
+      </c>
+      <c r="D2003" t="n">
+        <v>12572925524.81045</v>
+      </c>
+    </row>
+    <row r="2004">
+      <c r="A2004" t="inlineStr">
+        <is>
+          <t>ZWE</t>
+        </is>
+      </c>
+      <c r="B2004" t="inlineStr">
+        <is>
+          <t>Zimbabwe</t>
+        </is>
+      </c>
+      <c r="C2004" t="n">
+        <v>2008</v>
+      </c>
+      <c r="D2004" t="n">
+        <v>10351422061.70757</v>
+      </c>
+    </row>
+    <row r="2005">
+      <c r="A2005" t="inlineStr">
+        <is>
+          <t>ZWE</t>
+        </is>
+      </c>
+      <c r="B2005" t="inlineStr">
+        <is>
+          <t>Zimbabwe</t>
+        </is>
+      </c>
+      <c r="C2005" t="n">
+        <v>2009</v>
+      </c>
+      <c r="D2005" t="n">
+        <v>11595617444.66356</v>
+      </c>
+    </row>
+    <row r="2006">
+      <c r="A2006" t="inlineStr">
+        <is>
+          <t>ZWE</t>
+        </is>
+      </c>
+      <c r="B2006" t="inlineStr">
+        <is>
+          <t>Zimbabwe</t>
+        </is>
+      </c>
+      <c r="C2006" t="n">
+        <v>2010</v>
+      </c>
+      <c r="D2006" t="n">
+        <v>14083116362.76866</v>
+      </c>
+    </row>
+    <row r="2007">
+      <c r="A2007" t="inlineStr">
+        <is>
+          <t>ZWE</t>
+        </is>
+      </c>
+      <c r="B2007" t="inlineStr">
+        <is>
+          <t>Zimbabwe</t>
+        </is>
+      </c>
+      <c r="C2007" t="n">
+        <v>2011</v>
+      </c>
+      <c r="D2007" t="n">
+        <v>16142097162.99623</v>
+      </c>
+    </row>
+    <row r="2008">
+      <c r="A2008" t="inlineStr">
+        <is>
+          <t>ZWE</t>
+        </is>
+      </c>
+      <c r="B2008" t="inlineStr">
+        <is>
+          <t>Zimbabwe</t>
+        </is>
+      </c>
+      <c r="C2008" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D2008" t="n">
+        <v>18683650519.49866</v>
+      </c>
+    </row>
+    <row r="2009">
+      <c r="A2009" t="inlineStr">
+        <is>
+          <t>ZWE</t>
+        </is>
+      </c>
+      <c r="B2009" t="inlineStr">
+        <is>
+          <t>Zimbabwe</t>
+        </is>
+      </c>
+      <c r="C2009" t="n">
+        <v>2013</v>
+      </c>
+      <c r="D2009" t="n">
+        <v>19280916546.44884</v>
+      </c>
+    </row>
+    <row r="2010">
+      <c r="A2010" t="inlineStr">
+        <is>
+          <t>ZWE</t>
+        </is>
+      </c>
+      <c r="B2010" t="inlineStr">
+        <is>
+          <t>Zimbabwe</t>
+        </is>
+      </c>
+      <c r="C2010" t="n">
+        <v>2014</v>
+      </c>
+      <c r="D2010" t="n">
+        <v>19567149970.42023</v>
+      </c>
+    </row>
+    <row r="2011">
+      <c r="A2011" t="inlineStr">
+        <is>
+          <t>ZWE</t>
+        </is>
+      </c>
+      <c r="B2011" t="inlineStr">
+        <is>
+          <t>Zimbabwe</t>
+        </is>
+      </c>
+      <c r="C2011" t="n">
+        <v>2015</v>
+      </c>
+      <c r="D2011" t="n">
+        <v>19963120600</v>
+      </c>
+    </row>
+    <row r="2012">
+      <c r="A2012" t="inlineStr">
+        <is>
+          <t>ZWE</t>
+        </is>
+      </c>
+      <c r="B2012" t="inlineStr">
+        <is>
+          <t>Zimbabwe</t>
+        </is>
+      </c>
+      <c r="C2012" t="n">
+        <v>2016</v>
+      </c>
+      <c r="D2012" t="n">
+        <v>20142979412.31727</v>
+      </c>
+    </row>
+    <row r="2013">
+      <c r="A2013" t="inlineStr">
+        <is>
+          <t>ZWE</t>
+        </is>
+      </c>
+      <c r="B2013" t="inlineStr">
+        <is>
+          <t>Zimbabwe</t>
+        </is>
+      </c>
+      <c r="C2013" t="n">
+        <v>2017</v>
+      </c>
+      <c r="D2013" t="n">
+        <v>20964866130.33335</v>
+      </c>
+    </row>
+    <row r="2014">
+      <c r="A2014" t="inlineStr">
+        <is>
+          <t>ZWE</t>
+        </is>
+      </c>
+      <c r="B2014" t="inlineStr">
+        <is>
+          <t>Zimbabwe</t>
+        </is>
+      </c>
+      <c r="C2014" t="n">
+        <v>2018</v>
+      </c>
+      <c r="D2014" t="n">
+        <v>22015177994.7607</v>
+      </c>
+    </row>
+    <row r="2015">
+      <c r="A2015" t="inlineStr">
+        <is>
+          <t>ZWE</t>
+        </is>
+      </c>
+      <c r="B2015" t="inlineStr">
+        <is>
+          <t>Zimbabwe</t>
+        </is>
+      </c>
+      <c r="C2015" t="n">
+        <v>2019</v>
+      </c>
+      <c r="D2015" t="n">
+        <v>20621078642.74352</v>
+      </c>
+    </row>
+    <row r="2016">
+      <c r="A2016" t="inlineStr">
+        <is>
+          <t>ZWE</t>
+        </is>
+      </c>
+      <c r="B2016" t="inlineStr">
+        <is>
+          <t>Zimbabwe</t>
+        </is>
+      </c>
+      <c r="C2016" t="n">
+        <v>2020</v>
+      </c>
+      <c r="D2016" t="n">
+        <v>19009139108.24475</v>
+      </c>
+    </row>
+    <row r="2017">
+      <c r="A2017" t="inlineStr">
+        <is>
+          <t>ZWE</t>
+        </is>
+      </c>
+      <c r="B2017" t="inlineStr">
+        <is>
+          <t>Zimbabwe</t>
+        </is>
+      </c>
+      <c r="C2017" t="n">
+        <v>2021</v>
+      </c>
+      <c r="D2017" t="n">
+        <v>20618836222.17532</v>
+      </c>
+    </row>
+    <row r="2018">
+      <c r="A2018" t="inlineStr">
+        <is>
+          <t>ZWE</t>
+        </is>
+      </c>
+      <c r="B2018" t="inlineStr">
+        <is>
+          <t>Zimbabwe</t>
+        </is>
+      </c>
+      <c r="C2018" t="n">
+        <v>2022</v>
+      </c>
+      <c r="D2018" t="n">
         <v>21963674100.4816</v>
       </c>
     </row>

</xml_diff>